<commit_message>
Standardize test suite to use QaaS.Common.Assertions built-in hooks and minimize custom assertions
</commit_message>
<xml_diff>
--- a/tests_specification.xlsx
+++ b/tests_specification.xlsx
@@ -553,17 +553,17 @@
       </c>
       <c r="E2" s="5" t="inlineStr">
         <is>
-          <t>FireflyExpert records preserving all 12 input fields, correctly calculating: favorite_technology, favorite_team, favorite_commander, favorite_woman (lucky % 5), favorite_coding_language (by age), and base glow (height + 0.5*weight + lucky%10).</t>
+          <t>FireflyExpert records preserving all 12 input fields, correctly calculating: favorite_technology, favorite_team, favorite_commander, favorite_woman (lucky % 5), favorite_coding_language (by age), base glow, and mock comedic buff.</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>Verifies that Mamtzetza preserves input soldier identity and deterministically computes all 5 new firefly specialization attributes according to business specifications.</t>
+          <t>Verifies that Mamtzetza preserves input soldier identity and deterministically computes all 5 specialization attributes according to business logic.</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Custom QaaS Assertion: FireflyLogicalAssertion. Validates modulo rules, string parsing, and range lookups.</t>
+          <t>Custom QaaS Hook: FireflyLogicalAssertion (domain logic verification).</t>
         </is>
       </c>
     </row>
@@ -575,32 +575,32 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>ExternalApiEnrichment</t>
+          <t>OutputContractValidation</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>Integration / Mocking</t>
+          <t>Contract Validation / Schema</t>
         </is>
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t>OmegaSolider messages with ENABLE_EXTERNAL_API=true configured to query HTTP Mocker.</t>
+          <t>Raw binary byte stream consumed from RabbitMQ exchange firefly-expert-output.</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>FireflyExpert messages with bonusGlow (+50) added to glow_intensity and comedic_buff formatted as '{buffName} - {title}' via GET /api/v1/buff/{id} and POST /api/v1/funny-title.</t>
+          <t>Output payload cleanly deserializes to OmegaSolider.Messages.FireflyExpert Protobuf message contract with valid schema structure.</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>Validates dual-endpoint external HTTP REST mocking integration with QaaS Mocker, ensuring both buff retrieval and dynamic comedic title assignment succeed.</t>
+          <t>Validates contract compliance and serialization integrity across the wire using QaaS.Common.Assertions OutputDeserializableTo.</t>
         </is>
       </c>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t>Custom QaaS Assertion: FireflyApiEnrichmentAssertion. Confirms mock response parsing and attribute blending.</t>
+          <t>Built-in QaaS Hook: OutputDeserializableTo (QaaS.Common.Assertions).</t>
         </is>
       </c>
     </row>
@@ -612,32 +612,32 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>ExternalApiFallback</t>
+          <t>ExpectedBatchOutputCount</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Fault Tolerance / Resilience</t>
+          <t>Stress / Batch Integrity</t>
         </is>
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>OmegaSolider messages processed when external API is unreachable, degraded, or disabled.</t>
+          <t>Stream of messages published to RabbitMQ input exchange.</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
         <is>
-          <t>Valid FireflyExpert records emitted without exception. ComedicBuff gracefully degrades to 'API Error Fallback: ...' or 'Unbuffed Normal Firefly (No API)' without message dropping.</t>
+          <t>Exactly 5 output records are consumed by FireflyConsumer without queue truncation or buffer drops.</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Verifies component resilience and error handling, confirming Mamtzetza does not crash or poison queues when external microservices fail.</t>
+          <t>Verifies exact batch output quantity matching using QaaS.Common.Assertions HermeticByExpectedOutputCount.</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Custom QaaS Assertion: FireflyFallbackAssertion. Ensures high service availability and graceful degradation.</t>
+          <t>Built-in QaaS Hook: HermeticByExpectedOutputCount (QaaS.Common.Assertions).</t>
         </is>
       </c>
     </row>
@@ -654,7 +654,7 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Reliability / Integrity</t>
+          <t>Reliability / Throughput</t>
         </is>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -669,12 +669,12 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>Validates complete hermetic end-to-end processing across the RabbitMQ messaging topology using QaaS HermeticByInputOutputPercentage.</t>
+          <t>Validates complete hermetic end-to-end processing across the RabbitMQ messaging topology using QaaS.Common.Assertions HermeticByInputOutputPercentage.</t>
         </is>
       </c>
       <c r="G5" s="9" t="inlineStr">
         <is>
-          <t>Built-in QaaS Assertion: HermeticByInputOutputPercentage. ExpectedPercentage = 100%.</t>
+          <t>Built-in QaaS Hook: HermeticByInputOutputPercentage (QaaS.Common.Assertions).</t>
         </is>
       </c>
     </row>
@@ -686,12 +686,12 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>MaxProcessingDelay</t>
+          <t>MaxProcessingDelayByChunks</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Performance / SLA</t>
+          <t>Performance / Latency SLA</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
@@ -711,7 +711,7 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Built-in QaaS Assertion: DelayByChunks. ChunkSize = 1, MaximumDelayMs = 10000.</t>
+          <t>Built-in QaaS Hook: DelayByChunks (QaaS.Common.Assertions).</t>
         </is>
       </c>
     </row>
@@ -723,32 +723,32 @@
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>StressThroughputBurst</t>
+          <t>ProcessingDelayByAverage</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>Stress / Load</t>
+          <t>Performance / Average Latency</t>
         </is>
       </c>
       <c r="D7" s="9" t="inlineStr">
         <is>
-          <t>High-volume message burst published under peak throughput load to RabbitMQ.</t>
+          <t>End-to-end message flow published through the RabbitMQ and Mamtzetza pipeline.</t>
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr">
         <is>
-          <t>All messages processed and consumed without consumer stalling, buffer overflow, or channel timeout.</t>
+          <t>Average processing transit delay across all messages strictly under 5,000ms.</t>
         </is>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
-          <t>Stresses message deserialization, HTTP mock dispatching, and Protobuf serialization under load to verify component stability.</t>
+          <t>Measures and enforces average round-trip processing time using QaaS.Common.Assertions DelayByAverage.</t>
         </is>
       </c>
       <c r="G7" s="9" t="inlineStr">
         <is>
-          <t>Custom QaaS Assertion: FireflyStressAssertion. Validates queue drainage and memory stability.</t>
+          <t>Built-in QaaS Hook: DelayByAverage (QaaS.Common.Assertions).</t>
         </is>
       </c>
     </row>
@@ -765,7 +765,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>Observability / Metrics</t>
+          <t>Observability / Prometheus Metrics</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Custom QaaS Assertion: MamtzetzaMetricsAssertion. Scraped by Prometheus and visualized in monitoring dashboards.</t>
+          <t>Custom QaaS Hook: MamtzetzaMetricsAssertion (observability verification).</t>
         </is>
       </c>
     </row>
@@ -822,7 +822,7 @@
       </c>
       <c r="G9" s="9" t="inlineStr">
         <is>
-          <t>Custom QaaS Assertion: MamtzetzaLogsAssertion. Verifies JSON console formatting for centralized logging.</t>
+          <t>Custom QaaS Hook: MamtzetzaLogsAssertion (observability verification).</t>
         </is>
       </c>
     </row>

</xml_diff>